<commit_message>
Android App , Backend and Frontend are updated
</commit_message>
<xml_diff>
--- a/Backend/user_activity_logs.xlsx
+++ b/Backend/user_activity_logs.xlsx
@@ -518,27 +518,31 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-13 21:46:09</t>
+          <t>2026-03-31 12:50:24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-02-13 21:46:09</t>
+          <t>2026-03-31 12:50:24</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>47000143</t>
+          <t>abab279e</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>AGGREGATE, TREND</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-02-13 21:46:09</t>
+          <t>2026-03-31 12:50:24</t>
         </is>
       </c>
     </row>

</xml_diff>